<commit_message>
fix(privacy): replace personal sample data with dummy data and remove frontend API key inputs
</commit_message>
<xml_diff>
--- a/sample_data/bank_statement_sample.xlsx
+++ b/sample_data/bank_statement_sample.xlsx
@@ -417,69 +417,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr"/>
       <c r="B1" t="inlineStr">
         <is>
           <t>Account Statement</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ANIKET BALASAHEB GUND</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>RAHUL ARUN SHARMA</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Cust. Reln. No.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>987654321</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A-WING ,FLAT 11RAJHANS SOCIETY</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>FLAT 402, LOTUS RESIDENCY</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Account No.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>XXXXXX1234</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SEASONS ROAD</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>BANER ROAD</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>Period</t>
@@ -490,7 +473,6 @@
           <t>From 01/10/2026 To 26/10/2026</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -498,11 +480,6 @@
           <t>.</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Currency</t>
@@ -513,7 +490,6 @@
           <t>INR</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -521,11 +497,6 @@
           <t>PUNE</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Branch</t>
@@ -533,10 +504,9 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>AUNDAH, PUNE</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>BANER, PUNE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -544,11 +514,6 @@
           <t>MAHARASHTRA</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Nomination Regd</t>
@@ -559,7 +524,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -567,68 +531,49 @@
           <t>INDIA</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Nominee Name</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>411007</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+          <t>411045</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>Joint Holder(s)</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>IFSC</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>HDFC0001234</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>MICR</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-    </row>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>411240012</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -682,7 +627,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>01-10-2026 15:16</t>
+          <t>01-10-2026 09:15</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -692,17 +637,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>UPI/Maharashtra xe/YESB/061495859315/Payment from</t>
+          <t>UPI/STARBUCKS COFFEE/HDFC/992817263541/COFFEE</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>UPI-627415514786</t>
+          <t>UPI-718291029384</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>280.00</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -712,7 +657,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>39.7</t>
+          <t>4,970.00</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -727,7 +672,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>01-10-2026 20:05</t>
+          <t>01-10-2026 14:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -737,17 +682,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>UPI/Mrs MANGAL DAT/MAHB/339661873411/Payment from</t>
+          <t>UPI/SHREE GANESH TEA/YESB/112233445566/Payment from</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>UPI-627440723196</t>
+          <t>UPI-718291029385</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -757,7 +702,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>4,950.00</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -772,37 +717,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>04-10-2026 19:24</t>
+          <t>02-10-2026 11:20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>04-10-2026</t>
+          <t>02-10-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>UPI/BALASAHEB HARI/SBIN/211973126235/Payment from</t>
+          <t>UPI/PUNE METRO/HDFC/334455667788/TICKET</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>UPI-627766674481</t>
+          <t>UPI-718291029386</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>12,000.00</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>12,009.70</t>
+          <t>4,920.00</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -817,37 +762,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>04-10-2026 19:35</t>
+          <t>03-10-2026 19:40</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>04-10-2026</t>
+          <t>03-10-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>UPI/Dhruv /MAHG/130720604251/PAY BY WHATS</t>
+          <t>UPI/SHREE GANESH TEA/YESB/112233445566/Payment from</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>UPI-627767772666</t>
+          <t>UPI-718291029387</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2,420.00</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>14,429.70</t>
+          <t>4,900.00</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -862,7 +807,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>04-10-2026 19:58</t>
+          <t>04-10-2026 09:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -872,27 +817,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>UPI/KAUSTUBH SANJA/BARB/839588788818/Payment from</t>
+          <t>NEFT/INFOSYS TECHNOLOGIES/SALARY FOR OCT 2026/INF882910</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>UPI-627770425034</t>
+          <t>NEFT-88992019</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>65,000.00</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>DR</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>14,129.70</t>
+          <t>69,900.00</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -907,7 +852,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>04-10-2026 20:14</t>
+          <t>04-10-2026 11:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -917,17 +862,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>UPI/KAUSTUBH SANJA/BARB/892954188511/Payment from</t>
+          <t>UPI/SUNIL JOSHI/BARB/992211002211/OCTOBER HOUSE RENT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>UPI-627772041542</t>
+          <t>UPI-718291029388</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>18,000.00</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -937,7 +882,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14,029.70</t>
+          <t>51,900.00</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -952,7 +897,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>04-10-2026 21:21</t>
+          <t>04-10-2026 16:15</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -962,27 +907,27 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>UPI/NIKHIL SANTOSH/ICIC/811481986816/Payment from</t>
+          <t>UPI/ZERODHA BROKING/HDFC/554433221100/NIFTY50 SIP</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>UPI-627777916792</t>
+          <t>UPI-718291029389</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>4,800.00</t>
+          <t>5,000.00</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>18,829.70</t>
+          <t>46,900.00</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -997,27 +942,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>04-10-2026 23:00</t>
+          <t>05-10-2026 12:45</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>04-10-2026</t>
+          <t>05-10-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>UPI/MR ANIKET BALA/NESF/627786504949/SRe1f1b78532</t>
+          <t>UPI/D-MART BANER/YESB/778899001122/GROCERIES</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>UPI-627784737170</t>
+          <t>UPI-718291029390</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>18,800.00</t>
+          <t>3,450.00</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1027,7 +972,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>43,450.00</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1042,7 +987,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>05-10-2026 09:48</t>
+          <t>05-10-2026 20:10</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1052,27 +997,27 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>UPI/ATHRAV ADINATH/IPOS/627800410368/UPI</t>
+          <t>UPI/ZOMATO BANER/HDFC/445566778899/DINNER ORDER</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>UPI-627800732160</t>
+          <t>UPI-718291029391</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>4,800.00</t>
+          <t>420.00</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>4,829.70</t>
+          <t>43,030.00</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1087,37 +1032,37 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>05-10-2026 17:16</t>
+          <t>06-10-2026 10:20</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>05-10-2026</t>
+          <t>06-10-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>UPI/Dhruv /MAHG/130765891925/PAY BY WHATS</t>
+          <t>UPI/PUNE METRO/HDFC/334455667788/TICKET</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>UPI-627831531395</t>
+          <t>UPI-718291029392</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>5,379.70</t>
+          <t>43,000.00</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1132,37 +1077,37 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>05-10-2026 20:12</t>
+          <t>07-10-2026 15:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>05-10-2026</t>
+          <t>07-10-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>UPI/Dhruv /MAHG/130779376777/PAY BY WHATS</t>
+          <t>UPI/AIRTEL FIBER/AIRT/667788990011/BROADBAND BILL</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>UPI-627847852959</t>
+          <t>UPI-718291029393</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>4,800.00</t>
+          <t>999.00</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>10,179.70</t>
+          <t>42,001.00</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1177,37 +1122,37 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>05-10-2026 22:06</t>
+          <t>08-10-2026 11:15</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>05-10-2026</t>
+          <t>08-10-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>UPI/MR ANIKET BALA/NESF/627811747658/self transfe</t>
+          <t>UPI/MSEDCL ELECTRICITY/MAHA/889900112233/ELECTRICITY BILL</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>UPI-627857945340</t>
+          <t>UPI-718291029394</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>18,050.00</t>
+          <t>1,850.00</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>28,229.70</t>
+          <t>40,151.00</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1222,27 +1167,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>05-10-2026 22:07</t>
+          <t>09-10-2026 18:30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>05-10-2026</t>
+          <t>09-10-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>UPI/KALPANA SHARAD/BARB/695988802902/Payment from</t>
+          <t>UPI/AMAZON SELLER BANER/AMZN/990011223344/ELECTRONICS</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>UPI-627858046095</t>
+          <t>UPI-718291029395</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>24,000.00</t>
+          <t>2,199.00</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1252,7 +1197,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4,229.70</t>
+          <t>37,952.00</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1267,27 +1212,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>05-10-2026 22:12</t>
+          <t>10-10-2026 13:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>05-10-2026</t>
+          <t>10-10-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>UPI/slice/NESF/627863625774/UPI</t>
+          <t>UPI/SWIGGY FOOD/ICIC/110022993388/LUNCH ORDER</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>UPI-627858326187</t>
+          <t>UPI-718291029396</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1,686.24</t>
+          <t>380.00</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1297,7 +1242,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2,543.46</t>
+          <t>37,572.00</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1312,27 +1257,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>05-10-2026 22:25</t>
+          <t>11-10-2026 17:45</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>05-10-2026</t>
+          <t>11-10-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>UPI/slice/NESF/627885399193/UPI</t>
+          <t>UPI/UBER INDIA/ICIC/221133445566/CAB RIDE BANER</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>UPI-627859229645</t>
+          <t>UPI-718291029397</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>280.00</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1342,7 +1287,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1,793.46</t>
+          <t>37,292.00</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1357,27 +1302,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>05-10-2026 22:29</t>
+          <t>12-10-2026 10:10</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>05-10-2026</t>
+          <t>12-10-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>UPI/MR ANIKET BALA/NESF/627889870178/SR7343a0df50</t>
+          <t>UPI/APOLLO PHARMACY/YESB/332211445566/MEDICINES</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>UPI-627859492294</t>
+          <t>UPI-718291029398</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>793</t>
+          <t>650.00</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1387,7 +1332,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1,000.46</t>
+          <t>36,642.00</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1402,27 +1347,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06-10-2026 20:01</t>
+          <t>13-10-2026 19:20</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>06-10-2026</t>
+          <t>13-10-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>UPI/NAUSHAD SHARIF/YESB/804157419485/Payment from</t>
+          <t>UPI/NETFLIX INDIA/NETF/443322110099/SUBSCRIPTION</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>UPI-627920036089</t>
+          <t>UPI-718291029399</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>649.00</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1432,7 +1377,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>800.46</t>
+          <t>35,993.00</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1447,27 +1392,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07-10-2026 11:20</t>
+          <t>14-10-2026 21:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>07-10-2026</t>
+          <t>14-10-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>UPI/Maharashtra xe/YESB/819165297656/Payment from</t>
+          <t>UPI/HDFC CREDIT CARD/HDFC/556677889900/CARD PAYMENT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>UPI-628054052848</t>
+          <t>UPI-718291029400</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>4,800.00</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1477,7 +1422,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>775.46</t>
+          <t>31,193.00</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1492,37 +1437,37 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>07-10-2026 11:43</t>
+          <t>15-10-2026 14:15</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>07-10-2026</t>
+          <t>15-10-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>UPI/ONE PUNE NCMC /HDFC/825622743101/payment</t>
+          <t>UPI/AMIT PATEL/SBIN/667788112233/DINNER SHARE</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>UPI-628055548883</t>
+          <t>UPI-718291029401</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1,200.00</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>DR</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>745.46</t>
+          <t>32,393.00</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1537,27 +1482,27 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>07-10-2026 13:30</t>
+          <t>16-10-2026 11:30</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>07-10-2026</t>
+          <t>16-10-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>UPI/ONE PUNE NCMC /HDFC/650662763156/payment</t>
+          <t>UPI/INDIAN OIL BANER/IOCL/778899223344/PETROL</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>UPI-628062831568</t>
+          <t>UPI-718291029402</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1,500.00</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1567,7 +1512,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>715.46</t>
+          <t>30,893.00</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1582,27 +1527,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10-10-2026 16:01</t>
+          <t>17-10-2026 16:45</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10-10-2026</t>
+          <t>17-10-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>UPI/AMBIKA SUPER M/YESB/440301208137/Payment from</t>
+          <t>UPI/KIRANA CORNER/YESB/889900334455/DAIRY MILK</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>UPI-628397916943</t>
+          <t>UPI-718291029403</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1612,7 +1557,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>695.46</t>
+          <t>30,853.00</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1627,27 +1572,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>11-10-2026 18:08</t>
+          <t>18-10-2026 12:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11-10-2026</t>
+          <t>18-10-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>UPI/SARIKA ASHWIN /YESB/374085106667/Payment from</t>
+          <t>UPI/CAFE COFFEE DAY/HDFC/990011445566/SNACKS</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>UPI-628481594837</t>
+          <t>UPI-718291029404</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>150.00</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1657,7 +1602,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>675.46</t>
+          <t>30,703.00</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1672,27 +1617,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11-10-2026 18:22</t>
+          <t>18-10-2026 12:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>11-10-2026</t>
+          <t>18-10-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>UPI/Diamond Watch /YESB/508995645567/Payment from</t>
+          <t>UPI/CAFE COFFEE DAY/HDFC/990011445566/SNACKS</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>UPI-628482863812</t>
+          <t>UPI-718291029404</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>150.00</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1702,7 +1647,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>655.46</t>
+          <t>30,553.00</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -1717,33 +1662,37 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>12-10-2026 12:11</t>
+          <t>20-10-2026 18:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>12-10-2026</t>
+          <t>20-10-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CHRG:SMS ALERT FEE FOR THE MONTH OF SEP26</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
+          <t>UPI/TECHCORP INDIA/ICIC/112233556677/TRAVEL REIMBURSEMENT</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>UPI-718291029406</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>3,500.00</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>DR</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>652.98</t>
+          <t>34,053.00</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -1758,27 +1707,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>12-10-2026 20:11</t>
+          <t>21-10-2026 12:10</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>12-10-2026</t>
+          <t>21-10-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>UPI/NEHA CAFE/YESB/059549036428/Payment from</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>UPI-628564230397</t>
+          <t>CHRG:CONSOLIDATED SMS ALERT CHARGES Q3</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>17.70</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1788,7 +1732,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>592.98</t>
+          <t>34,035.30</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">

</xml_diff>